<commit_message>
fix(tracker): use same-sheet reference in deal-age highlight rule
Google Sheets does not support cross-sheet references in conditional
formatting, so the stale-deal highlight on ดีลในมือ silently broke on
import. Compute the threshold into a helper cell on that sheet and point
the rule at it.

Also allow the start date, day count, and output path to be overridden
with env vars so a smaller workbook can be generated for verification.
</commit_message>
<xml_diff>
--- a/docs/investment-plan/home2hatyai-plan-tracker.xlsx
+++ b/docs/investment-plan/home2hatyai-plan-tracker.xlsx
@@ -194,7 +194,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="68">
+  <cellXfs count="69">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -314,6 +314,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="9" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -15687,6 +15690,15 @@
       </c>
       <c r="M16" s="26" t="n"/>
       <c r="N16" s="37" t="n"/>
+      <c r="P16" s="32" t="inlineStr">
+        <is>
+          <t>เกณฑ์ดีลค้างนาน (วัน)</t>
+        </is>
+      </c>
+      <c r="Q16" s="41">
+        <f>ROUND('ตั้งค่า'!$C$15*1.5,0)</f>
+        <v/>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="35" t="n"/>
@@ -17254,7 +17266,7 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="L7:L66">
     <cfRule type="cellIs" priority="3" operator="greaterThan" dxfId="7">
-      <formula>'ตั้งค่า'!$C$15*1.5</formula>
+      <formula>$Q$16</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
@@ -17365,7 +17377,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="41" t="n">
+      <c r="A4" s="42" t="n">
         <v>0</v>
       </c>
       <c r="B4" s="26" t="inlineStr">
@@ -17401,7 +17413,7 @@
         <f>IFERROR($F4/$F$24,"")</f>
         <v/>
       </c>
-      <c r="J4" s="42" t="n">
+      <c r="J4" s="43" t="n">
         <v>0.015</v>
       </c>
       <c r="K4" s="17" t="inlineStr">
@@ -17411,7 +17423,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="41" t="n">
+      <c r="A5" s="42" t="n">
         <v>0</v>
       </c>
       <c r="B5" s="26" t="inlineStr">
@@ -17447,7 +17459,7 @@
         <f>IFERROR($F5/$F$24,"")</f>
         <v/>
       </c>
-      <c r="J5" s="42" t="n">
+      <c r="J5" s="43" t="n">
         <v>0.018</v>
       </c>
       <c r="K5" s="17" t="inlineStr">
@@ -17457,7 +17469,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="41" t="n">
+      <c r="A6" s="42" t="n">
         <v>1</v>
       </c>
       <c r="B6" s="26" t="inlineStr">
@@ -17493,7 +17505,7 @@
         <f>IFERROR($F6/$F$24,"")</f>
         <v/>
       </c>
-      <c r="J6" s="42" t="n">
+      <c r="J6" s="43" t="n">
         <v>0.025</v>
       </c>
       <c r="K6" s="17" t="inlineStr">
@@ -17503,7 +17515,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="41" t="n">
+      <c r="A7" s="42" t="n">
         <v>1</v>
       </c>
       <c r="B7" s="26" t="inlineStr">
@@ -17539,7 +17551,7 @@
         <f>IFERROR($F7/$F$24,"")</f>
         <v/>
       </c>
-      <c r="J7" s="42" t="n">
+      <c r="J7" s="43" t="n">
         <v>0.022</v>
       </c>
       <c r="K7" s="17" t="inlineStr">
@@ -17549,7 +17561,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="41" t="n">
+      <c r="A8" s="42" t="n">
         <v>2</v>
       </c>
       <c r="B8" s="26" t="inlineStr">
@@ -17585,7 +17597,7 @@
         <f>IFERROR($F8/$F$24,"")</f>
         <v/>
       </c>
-      <c r="J8" s="42" t="n">
+      <c r="J8" s="43" t="n">
         <v>0.045</v>
       </c>
       <c r="K8" s="17" t="inlineStr">
@@ -17595,7 +17607,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="41" t="n">
+      <c r="A9" s="42" t="n">
         <v>2</v>
       </c>
       <c r="B9" s="26" t="inlineStr">
@@ -17631,7 +17643,7 @@
         <f>IFERROR($F9/$F$24,"")</f>
         <v/>
       </c>
-      <c r="J9" s="42" t="n">
+      <c r="J9" s="43" t="n">
         <v>0.055</v>
       </c>
       <c r="K9" s="17" t="inlineStr">
@@ -17641,7 +17653,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="41" t="n">
+      <c r="A10" s="42" t="n">
         <v>3</v>
       </c>
       <c r="B10" s="26" t="inlineStr">
@@ -17677,7 +17689,7 @@
         <f>IFERROR($F10/$F$24,"")</f>
         <v/>
       </c>
-      <c r="J10" s="42" t="n">
+      <c r="J10" s="43" t="n">
         <v>0.075</v>
       </c>
       <c r="K10" s="17" t="inlineStr">
@@ -17687,7 +17699,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="41" t="n">
+      <c r="A11" s="42" t="n">
         <v>3</v>
       </c>
       <c r="B11" s="26" t="inlineStr">
@@ -17723,7 +17735,7 @@
         <f>IFERROR($F11/$F$24,"")</f>
         <v/>
       </c>
-      <c r="J11" s="42" t="n">
+      <c r="J11" s="43" t="n">
         <v>0.06</v>
       </c>
       <c r="K11" s="17" t="inlineStr">
@@ -17733,7 +17745,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="41" t="n">
+      <c r="A12" s="42" t="n">
         <v>4</v>
       </c>
       <c r="B12" s="26" t="inlineStr">
@@ -17769,7 +17781,7 @@
         <f>IFERROR($F12/$F$24,"")</f>
         <v/>
       </c>
-      <c r="J12" s="42" t="n">
+      <c r="J12" s="43" t="n">
         <v>0.07000000000000001</v>
       </c>
       <c r="K12" s="17" t="inlineStr">
@@ -17779,7 +17791,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="41" t="n">
+      <c r="A13" s="42" t="n">
         <v>4</v>
       </c>
       <c r="B13" s="26" t="inlineStr">
@@ -17815,7 +17827,7 @@
         <f>IFERROR($F13/$F$24,"")</f>
         <v/>
       </c>
-      <c r="J13" s="42" t="n">
+      <c r="J13" s="43" t="n">
         <v>0.07000000000000001</v>
       </c>
       <c r="K13" s="17" t="inlineStr">
@@ -17825,7 +17837,7 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="41" t="n"/>
+      <c r="A14" s="42" t="n"/>
       <c r="B14" s="26" t="n"/>
       <c r="C14" s="26" t="n"/>
       <c r="D14" s="35" t="n"/>
@@ -17843,11 +17855,11 @@
         <f>IFERROR($F14/$F$24,"")</f>
         <v/>
       </c>
-      <c r="J14" s="42" t="n"/>
+      <c r="J14" s="43" t="n"/>
       <c r="K14" s="17" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="41" t="n"/>
+      <c r="A15" s="42" t="n"/>
       <c r="B15" s="26" t="n"/>
       <c r="C15" s="26" t="n"/>
       <c r="D15" s="35" t="n"/>
@@ -17865,11 +17877,11 @@
         <f>IFERROR($F15/$F$24,"")</f>
         <v/>
       </c>
-      <c r="J15" s="42" t="n"/>
+      <c r="J15" s="43" t="n"/>
       <c r="K15" s="17" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="41" t="n"/>
+      <c r="A16" s="42" t="n"/>
       <c r="B16" s="26" t="n"/>
       <c r="C16" s="26" t="n"/>
       <c r="D16" s="35" t="n"/>
@@ -17887,11 +17899,11 @@
         <f>IFERROR($F16/$F$24,"")</f>
         <v/>
       </c>
-      <c r="J16" s="42" t="n"/>
+      <c r="J16" s="43" t="n"/>
       <c r="K16" s="17" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="41" t="n"/>
+      <c r="A17" s="42" t="n"/>
       <c r="B17" s="26" t="n"/>
       <c r="C17" s="26" t="n"/>
       <c r="D17" s="35" t="n"/>
@@ -17909,11 +17921,11 @@
         <f>IFERROR($F17/$F$24,"")</f>
         <v/>
       </c>
-      <c r="J17" s="42" t="n"/>
+      <c r="J17" s="43" t="n"/>
       <c r="K17" s="17" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="41" t="n"/>
+      <c r="A18" s="42" t="n"/>
       <c r="B18" s="26" t="n"/>
       <c r="C18" s="26" t="n"/>
       <c r="D18" s="35" t="n"/>
@@ -17931,11 +17943,11 @@
         <f>IFERROR($F18/$F$24,"")</f>
         <v/>
       </c>
-      <c r="J18" s="42" t="n"/>
+      <c r="J18" s="43" t="n"/>
       <c r="K18" s="17" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="41" t="n"/>
+      <c r="A19" s="42" t="n"/>
       <c r="B19" s="26" t="n"/>
       <c r="C19" s="26" t="n"/>
       <c r="D19" s="35" t="n"/>
@@ -17953,11 +17965,11 @@
         <f>IFERROR($F19/$F$24,"")</f>
         <v/>
       </c>
-      <c r="J19" s="42" t="n"/>
+      <c r="J19" s="43" t="n"/>
       <c r="K19" s="17" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="41" t="n"/>
+      <c r="A20" s="42" t="n"/>
       <c r="B20" s="26" t="n"/>
       <c r="C20" s="26" t="n"/>
       <c r="D20" s="35" t="n"/>
@@ -17975,11 +17987,11 @@
         <f>IFERROR($F20/$F$24,"")</f>
         <v/>
       </c>
-      <c r="J20" s="42" t="n"/>
+      <c r="J20" s="43" t="n"/>
       <c r="K20" s="17" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="41" t="n"/>
+      <c r="A21" s="42" t="n"/>
       <c r="B21" s="26" t="n"/>
       <c r="C21" s="26" t="n"/>
       <c r="D21" s="35" t="n"/>
@@ -17997,11 +18009,11 @@
         <f>IFERROR($F21/$F$24,"")</f>
         <v/>
       </c>
-      <c r="J21" s="42" t="n"/>
+      <c r="J21" s="43" t="n"/>
       <c r="K21" s="17" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="41" t="n"/>
+      <c r="A22" s="42" t="n"/>
       <c r="B22" s="26" t="n"/>
       <c r="C22" s="26" t="n"/>
       <c r="D22" s="35" t="n"/>
@@ -18019,11 +18031,11 @@
         <f>IFERROR($F22/$F$24,"")</f>
         <v/>
       </c>
-      <c r="J22" s="42" t="n"/>
+      <c r="J22" s="43" t="n"/>
       <c r="K22" s="17" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="41" t="n"/>
+      <c r="A23" s="42" t="n"/>
       <c r="B23" s="26" t="n"/>
       <c r="C23" s="26" t="n"/>
       <c r="D23" s="35" t="n"/>
@@ -18041,47 +18053,47 @@
         <f>IFERROR($F23/$F$24,"")</f>
         <v/>
       </c>
-      <c r="J23" s="42" t="n"/>
+      <c r="J23" s="43" t="n"/>
       <c r="K23" s="17" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="43" t="inlineStr">
+      <c r="A24" s="44" t="inlineStr">
         <is>
           <t>รวม</t>
         </is>
       </c>
-      <c r="B24" s="44" t="inlineStr">
+      <c r="B24" s="45" t="inlineStr">
         <is>
           <t>พอร์ตทั้งหมด</t>
         </is>
       </c>
-      <c r="C24" s="45" t="n"/>
-      <c r="D24" s="45" t="n"/>
-      <c r="E24" s="46">
+      <c r="C24" s="46" t="n"/>
+      <c r="D24" s="46" t="n"/>
+      <c r="E24" s="47">
         <f>SUM(E4:E23)</f>
         <v/>
       </c>
-      <c r="F24" s="46">
+      <c r="F24" s="47">
         <f>SUM(F4:F23)</f>
         <v/>
       </c>
-      <c r="G24" s="46">
+      <c r="G24" s="47">
         <f>F24-E24</f>
         <v/>
       </c>
-      <c r="H24" s="47">
+      <c r="H24" s="48">
         <f>IFERROR(G24/E24,"")</f>
         <v/>
       </c>
-      <c r="I24" s="47">
+      <c r="I24" s="48">
         <f>IFERROR(F24/F24,"")</f>
         <v/>
       </c>
-      <c r="J24" s="48">
+      <c r="J24" s="49">
         <f>IFERROR(SUMPRODUCT($F$4:$F$23,$J$4:$J$23)/$F$24,0)</f>
         <v/>
       </c>
-      <c r="K24" s="49" t="inlineStr">
+      <c r="K24" s="50" t="inlineStr">
         <is>
           <t>ผลตอบแทนคาดหวังถ่วงน้ำหนักของพอร์ตจริง</t>
         </is>
@@ -18135,7 +18147,7 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="50" t="n">
+      <c r="A28" s="51" t="n">
         <v>0</v>
       </c>
       <c r="B28" s="11" t="inlineStr">
@@ -18143,19 +18155,19 @@
           <t>เงินสำรองฉุกเฉิน (เงินสด)</t>
         </is>
       </c>
-      <c r="C28" s="51">
+      <c r="C28" s="52">
         <f>SUMIF($A$4:$A$23,0,$F$4:$F$23)</f>
         <v/>
       </c>
-      <c r="D28" s="52">
+      <c r="D28" s="53">
         <f>IFERROR(C28/$C$33,"")</f>
         <v/>
       </c>
-      <c r="E28" s="51">
+      <c r="E28" s="52">
         <f>'ตั้งค่า'!$C$31</f>
         <v/>
       </c>
-      <c r="F28" s="51">
+      <c r="F28" s="52">
         <f>E28-C28</f>
         <v/>
       </c>
@@ -18165,7 +18177,7 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="50" t="n">
+      <c r="A29" s="51" t="n">
         <v>1</v>
       </c>
       <c r="B29" s="11" t="inlineStr">
@@ -18173,19 +18185,19 @@
           <t>ปลอดภัย — พันธบัตร/ตราสารหนี้</t>
         </is>
       </c>
-      <c r="C29" s="51">
+      <c r="C29" s="52">
         <f>SUMIF($A$4:$A$23,1,$F$4:$F$23)</f>
         <v/>
       </c>
-      <c r="D29" s="52">
+      <c r="D29" s="53">
         <f>IFERROR(C29/$C$33,"")</f>
         <v/>
       </c>
-      <c r="E29" s="51">
+      <c r="E29" s="52">
         <f>MAX(0,$C$33-$E$28)*'ตั้งค่า'!$C$40</f>
         <v/>
       </c>
-      <c r="F29" s="51">
+      <c r="F29" s="52">
         <f>E29-C29</f>
         <v/>
       </c>
@@ -18195,7 +18207,7 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="50" t="n">
+      <c r="A30" s="51" t="n">
         <v>2</v>
       </c>
       <c r="B30" s="11" t="inlineStr">
@@ -18203,19 +18215,19 @@
           <t>รายได้ประจำ — หุ้นกู้/REIT</t>
         </is>
       </c>
-      <c r="C30" s="51">
+      <c r="C30" s="52">
         <f>SUMIF($A$4:$A$23,2,$F$4:$F$23)</f>
         <v/>
       </c>
-      <c r="D30" s="52">
+      <c r="D30" s="53">
         <f>IFERROR(C30/$C$33,"")</f>
         <v/>
       </c>
-      <c r="E30" s="51">
+      <c r="E30" s="52">
         <f>MAX(0,$C$33-$E$28)*'ตั้งค่า'!$C$41</f>
         <v/>
       </c>
-      <c r="F30" s="51">
+      <c r="F30" s="52">
         <f>E30-C30</f>
         <v/>
       </c>
@@ -18225,7 +18237,7 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="50" t="n">
+      <c r="A31" s="51" t="n">
         <v>3</v>
       </c>
       <c r="B31" s="11" t="inlineStr">
@@ -18233,19 +18245,19 @@
           <t>เติบโต — กองดัชนีหุ้น (DCA)</t>
         </is>
       </c>
-      <c r="C31" s="51">
+      <c r="C31" s="52">
         <f>SUMIF($A$4:$A$23,3,$F$4:$F$23)</f>
         <v/>
       </c>
-      <c r="D31" s="52">
+      <c r="D31" s="53">
         <f>IFERROR(C31/$C$33,"")</f>
         <v/>
       </c>
-      <c r="E31" s="51">
+      <c r="E31" s="52">
         <f>MAX(0,$C$33-$E$28)*'ตั้งค่า'!$C$42</f>
         <v/>
       </c>
-      <c r="F31" s="51">
+      <c r="F31" s="52">
         <f>E31-C31</f>
         <v/>
       </c>
@@ -18255,7 +18267,7 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="50" t="n">
+      <c r="A32" s="51" t="n">
         <v>4</v>
       </c>
       <c r="B32" s="11" t="inlineStr">
@@ -18263,19 +18275,19 @@
           <t>ลดหย่อนภาษี — Thai ESG/SSF/RMF</t>
         </is>
       </c>
-      <c r="C32" s="51">
+      <c r="C32" s="52">
         <f>SUMIF($A$4:$A$23,4,$F$4:$F$23)</f>
         <v/>
       </c>
-      <c r="D32" s="52">
+      <c r="D32" s="53">
         <f>IFERROR(C32/$C$33,"")</f>
         <v/>
       </c>
-      <c r="E32" s="51">
+      <c r="E32" s="52">
         <f>MAX(0,$C$33-$E$28)*'ตั้งค่า'!$C$43</f>
         <v/>
       </c>
-      <c r="F32" s="51">
+      <c r="F32" s="52">
         <f>E32-C32</f>
         <v/>
       </c>
@@ -18285,20 +18297,20 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="45" t="inlineStr"/>
-      <c r="B33" s="44" t="inlineStr">
+      <c r="A33" s="46" t="inlineStr"/>
+      <c r="B33" s="45" t="inlineStr">
         <is>
           <t>รวมทุกชั้น</t>
         </is>
       </c>
-      <c r="C33" s="46">
+      <c r="C33" s="47">
         <f>SUM(C28:C32)</f>
         <v/>
       </c>
-      <c r="D33" s="45" t="n"/>
-      <c r="E33" s="45" t="n"/>
-      <c r="F33" s="45" t="n"/>
-      <c r="G33" s="45" t="n"/>
+      <c r="D33" s="46" t="n"/>
+      <c r="E33" s="46" t="n"/>
+      <c r="F33" s="46" t="n"/>
+      <c r="G33" s="46" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -27351,7 +27363,7 @@
           <t>ราคาทรัพย์เฉลี่ยต่อดีล (บาท)</t>
         </is>
       </c>
-      <c r="C5" s="53" t="n">
+      <c r="C5" s="54" t="n">
         <v>2800000</v>
       </c>
       <c r="D5" s="17" t="inlineStr">
@@ -27366,7 +27378,7 @@
           <t>อัตราค่าคอมมิชชันที่ได้รับ (%)</t>
         </is>
       </c>
-      <c r="C6" s="54" t="n">
+      <c r="C6" s="55" t="n">
         <v>0.03</v>
       </c>
       <c r="D6" s="17" t="inlineStr">
@@ -27381,7 +27393,7 @@
           <t>ส่วนแบ่งให้ co-agent / ทีม (%)</t>
         </is>
       </c>
-      <c r="C7" s="54" t="n">
+      <c r="C7" s="55" t="n">
         <v>0</v>
       </c>
       <c r="D7" s="17" t="inlineStr">
@@ -27396,7 +27408,7 @@
           <t>➜ คอมมิชชันสุทธิต่อ 1 ดีล (บาท)</t>
         </is>
       </c>
-      <c r="C8" s="55">
+      <c r="C8" s="56">
         <f>$C$5*$C$6*(1-$C$7)</f>
         <v/>
       </c>
@@ -27412,7 +27424,7 @@
           <t>งบโฆษณาต่อวัน (บาท)</t>
         </is>
       </c>
-      <c r="C9" s="53" t="n">
+      <c r="C9" s="54" t="n">
         <v>500</v>
       </c>
       <c r="D9" s="17" t="inlineStr">
@@ -27427,7 +27439,7 @@
           <t>ต้นทุนคงที่ต่อเดือน (บาท)</t>
         </is>
       </c>
-      <c r="C10" s="53" t="n">
+      <c r="C10" s="54" t="n">
         <v>15000</v>
       </c>
       <c r="D10" s="17" t="inlineStr">
@@ -27442,7 +27454,7 @@
           <t>อัตราปิด: lead คุณภาพ ➜ โอน (%)</t>
         </is>
       </c>
-      <c r="C11" s="54" t="n">
+      <c r="C11" s="55" t="n">
         <v>0.03</v>
       </c>
       <c r="D11" s="17" t="inlineStr">
@@ -27457,7 +27469,7 @@
           <t>CPQL จริง — ค่าโฆษณาต่อ lead คุณภาพ 1 คน (บาท)</t>
         </is>
       </c>
-      <c r="C12" s="53" t="n">
+      <c r="C12" s="54" t="n">
         <v>400</v>
       </c>
       <c r="D12" s="17" t="inlineStr">
@@ -27472,7 +27484,7 @@
           <t>➜ มูลค่าของ lead คุณภาพ 1 คน (บาท)</t>
         </is>
       </c>
-      <c r="C13" s="55">
+      <c r="C13" s="56">
         <f>$C$8*$C$11</f>
         <v/>
       </c>
@@ -27488,7 +27500,7 @@
           <t>➜ เพดาน CPQL ที่ยอมจ่ายได้ (บาท)</t>
         </is>
       </c>
-      <c r="C14" s="55">
+      <c r="C14" s="56">
         <f>$C$13*0.25</f>
         <v/>
       </c>
@@ -27504,7 +27516,7 @@
           <t>จำนวนวันเฉลี่ย: lead ➜ โอนเงิน</t>
         </is>
       </c>
-      <c r="C15" s="53" t="n">
+      <c r="C15" s="54" t="n">
         <v>75</v>
       </c>
       <c r="D15" s="17" t="inlineStr">
@@ -27526,7 +27538,7 @@
           <t>เป้ารายได้ค่าคอมต่อเดือน (บาท)</t>
         </is>
       </c>
-      <c r="C17" s="53" t="n">
+      <c r="C17" s="54" t="n">
         <v>150000</v>
       </c>
       <c r="D17" s="17" t="inlineStr">
@@ -27541,7 +27553,7 @@
           <t>➜ ต้องปิดกี่ดีลต่อเดือน</t>
         </is>
       </c>
-      <c r="C18" s="56">
+      <c r="C18" s="57">
         <f>IFERROR($C$17/$C$8,0)</f>
         <v/>
       </c>
@@ -27553,7 +27565,7 @@
           <t>➜ ต้องมี lead คุณภาพกี่คนต่อเดือน</t>
         </is>
       </c>
-      <c r="C19" s="57">
+      <c r="C19" s="58">
         <f>IFERROR($C$18/$C$11,0)</f>
         <v/>
       </c>
@@ -27565,7 +27577,7 @@
           <t>➜ ต้องมี lead คุณภาพกี่คนต่อวัน</t>
         </is>
       </c>
-      <c r="C20" s="58">
+      <c r="C20" s="59">
         <f>IFERROR($C$19/30,0)</f>
         <v/>
       </c>
@@ -27581,7 +27593,7 @@
           <t>➜ งบโฆษณาต่อเดือน (บาท)</t>
         </is>
       </c>
-      <c r="C21" s="55">
+      <c r="C21" s="56">
         <f>$C$9*30</f>
         <v/>
       </c>
@@ -27593,7 +27605,7 @@
           <t>➜ lead คุณภาพที่งบนี้ควรได้ (คน/เดือน)</t>
         </is>
       </c>
-      <c r="C22" s="57">
+      <c r="C22" s="58">
         <f>IFERROR($C$21/$C$12,0)</f>
         <v/>
       </c>
@@ -27605,7 +27617,7 @@
           <t>➜ รายได้ที่คาดว่าจะได้ (บาท/เดือน)</t>
         </is>
       </c>
-      <c r="C23" s="55">
+      <c r="C23" s="56">
         <f>IFERROR($C$22*$C$11*$C$8,0)</f>
         <v/>
       </c>
@@ -27617,7 +27629,7 @@
           <t>➜ กำไรสุทธิที่คาดว่าจะได้ (บาท/เดือน)</t>
         </is>
       </c>
-      <c r="C24" s="55">
+      <c r="C24" s="56">
         <f>$C$23-$C$21-$C$10</f>
         <v/>
       </c>
@@ -27633,7 +27645,7 @@
           <t>➜ ROAS — ได้กี่เท่าของค่าโฆษณา</t>
         </is>
       </c>
-      <c r="C25" s="59">
+      <c r="C25" s="60">
         <f>IFERROR($C$23/$C$21,0)</f>
         <v/>
       </c>
@@ -27649,7 +27661,7 @@
           <t>➜ งบโฆษณาที่ควรใช้เพื่อถึงเป้า (บาท/เดือน)</t>
         </is>
       </c>
-      <c r="C26" s="55">
+      <c r="C26" s="56">
         <f>IFERROR($C$19*$C$12,0)</f>
         <v/>
       </c>
@@ -27672,7 +27684,7 @@
           <t>ทุนตั้งต้นที่มีตอนนี้ (บาท)</t>
         </is>
       </c>
-      <c r="C28" s="53" t="n">
+      <c r="C28" s="54" t="n">
         <v>100000</v>
       </c>
       <c r="D28" s="17" t="inlineStr">
@@ -27687,7 +27699,7 @@
           <t>รายจ่ายจำเป็นส่วนตัวต่อเดือน (บาท)</t>
         </is>
       </c>
-      <c r="C29" s="53" t="n">
+      <c r="C29" s="54" t="n">
         <v>25000</v>
       </c>
       <c r="D29" s="17" t="inlineStr">
@@ -27702,7 +27714,7 @@
           <t>จำนวนเดือนที่ต้องมีเงินสำรอง</t>
         </is>
       </c>
-      <c r="C30" s="53" t="n">
+      <c r="C30" s="54" t="n">
         <v>6</v>
       </c>
       <c r="D30" s="17" t="inlineStr">
@@ -27717,7 +27729,7 @@
           <t>➜ เงินสำรองฉุกเฉินเป้าหมาย (บาท)</t>
         </is>
       </c>
-      <c r="C31" s="55">
+      <c r="C31" s="56">
         <f>($C$29+$C$10)*$C$30</f>
         <v/>
       </c>
@@ -27733,7 +27745,7 @@
           <t>ฐานภาษีเงินได้สูงสุดของคุณ (%)</t>
         </is>
       </c>
-      <c r="C32" s="54" t="n">
+      <c r="C32" s="55" t="n">
         <v>0.2</v>
       </c>
       <c r="D32" s="17" t="inlineStr">
@@ -27755,7 +27767,7 @@
           <t>% เข้าบัญชีภาษี + เงินสำรอง</t>
         </is>
       </c>
-      <c r="C34" s="54" t="n">
+      <c r="C34" s="55" t="n">
         <v>0.3</v>
       </c>
       <c r="D34" s="17" t="inlineStr">
@@ -27770,7 +27782,7 @@
           <t>% เติมกลับเข้าโฆษณา (ขยายธุรกิจ)</t>
         </is>
       </c>
-      <c r="C35" s="54" t="n">
+      <c r="C35" s="55" t="n">
         <v>0.2</v>
       </c>
       <c r="D35" s="17" t="inlineStr">
@@ -27785,7 +27797,7 @@
           <t>% เข้าพอร์ตลงทุน</t>
         </is>
       </c>
-      <c r="C36" s="54" t="n">
+      <c r="C36" s="55" t="n">
         <v>0.3</v>
       </c>
       <c r="D36" s="17" t="inlineStr">
@@ -27800,7 +27812,7 @@
           <t>% ใช้จ่ายส่วนตัว</t>
         </is>
       </c>
-      <c r="C37" s="54" t="n">
+      <c r="C37" s="55" t="n">
         <v>0.2</v>
       </c>
       <c r="D37" s="17" t="inlineStr">
@@ -27815,7 +27827,7 @@
           <t>➜ รวม (ต้องได้ 100%)</t>
         </is>
       </c>
-      <c r="C38" s="60">
+      <c r="C38" s="61">
         <f>$C$34+$C$35+$C$36+$C$37</f>
         <v/>
       </c>
@@ -27838,7 +27850,7 @@
           <t>ชั้น 1 · ปลอดภัย (พันธบัตร / กองตราสารหนี้ / ฝากดอกสูง)</t>
         </is>
       </c>
-      <c r="C40" s="54" t="n">
+      <c r="C40" s="55" t="n">
         <v>0.4</v>
       </c>
       <c r="D40" s="17" t="inlineStr">
@@ -27853,7 +27865,7 @@
           <t>ชั้น 2 · รายได้ประจำ (หุ้นกู้เรตติ้งดี / REIT / กองปันผล)</t>
         </is>
       </c>
-      <c r="C41" s="54" t="n">
+      <c r="C41" s="55" t="n">
         <v>0.25</v>
       </c>
       <c r="D41" s="17" t="inlineStr">
@@ -27868,7 +27880,7 @@
           <t>ชั้น 3 · เติบโต (กองทุนดัชนีหุ้นโลก ทยอยซื้อ DCA)</t>
         </is>
       </c>
-      <c r="C42" s="54" t="n">
+      <c r="C42" s="55" t="n">
         <v>0.25</v>
       </c>
       <c r="D42" s="17" t="inlineStr">
@@ -27883,7 +27895,7 @@
           <t>ชั้น 4 · ลดหย่อนภาษี (Thai ESG / SSF / RMF)</t>
         </is>
       </c>
-      <c r="C43" s="54" t="n">
+      <c r="C43" s="55" t="n">
         <v>0.1</v>
       </c>
       <c r="D43" s="17" t="inlineStr">
@@ -27898,7 +27910,7 @@
           <t>➜ รวม (ต้องได้ 100%)</t>
         </is>
       </c>
-      <c r="C44" s="60">
+      <c r="C44" s="61">
         <f>$C$40+$C$41+$C$42+$C$43</f>
         <v/>
       </c>
@@ -27910,7 +27922,7 @@
           <t>ผลตอบแทนคาดหวังชั้น 1 (%/ปี)</t>
         </is>
       </c>
-      <c r="C45" s="54" t="n">
+      <c r="C45" s="55" t="n">
         <v>0.025</v>
       </c>
       <c r="D45" s="17" t="inlineStr"/>
@@ -27921,7 +27933,7 @@
           <t>ผลตอบแทนคาดหวังชั้น 2 (%/ปี)</t>
         </is>
       </c>
-      <c r="C46" s="54" t="n">
+      <c r="C46" s="55" t="n">
         <v>0.05</v>
       </c>
       <c r="D46" s="17" t="inlineStr"/>
@@ -27932,7 +27944,7 @@
           <t>ผลตอบแทนคาดหวังชั้น 3 (%/ปี)</t>
         </is>
       </c>
-      <c r="C47" s="54" t="n">
+      <c r="C47" s="55" t="n">
         <v>0.075</v>
       </c>
       <c r="D47" s="17" t="inlineStr"/>
@@ -27943,7 +27955,7 @@
           <t>ผลตอบแทนคาดหวังชั้น 4 (%/ปี)</t>
         </is>
       </c>
-      <c r="C48" s="54" t="n">
+      <c r="C48" s="55" t="n">
         <v>0.07000000000000001</v>
       </c>
       <c r="D48" s="17" t="inlineStr">
@@ -27958,7 +27970,7 @@
           <t>➜ ผลตอบแทนพอร์ตรวมที่คาดหวัง (%/ปี)</t>
         </is>
       </c>
-      <c r="C49" s="60">
+      <c r="C49" s="61">
         <f>($C$40*$C$45)+($C$41*$C$46)+($C$42*$C$47)+($C$43*$C$48)</f>
         <v/>
       </c>
@@ -27974,7 +27986,7 @@
           <t>➜ บวกผลจากภาษีคืนปีแรก (%/ปี)</t>
         </is>
       </c>
-      <c r="C50" s="60">
+      <c r="C50" s="61">
         <f>$C$49+($C$43*$C$32)</f>
         <v/>
       </c>
@@ -28061,15 +28073,15 @@
       </c>
     </row>
     <row r="4" ht="34" customHeight="1">
-      <c r="A4" s="50" t="n">
+      <c r="A4" s="51" t="n">
         <v>1</v>
       </c>
-      <c r="B4" s="61" t="inlineStr">
+      <c r="B4" s="62" t="inlineStr">
         <is>
           <t>ห้ามลงทุนด้วยเงินที่ต้องใช้ภายใน 12 เดือน</t>
         </is>
       </c>
-      <c r="C4" s="62" t="inlineStr">
+      <c r="C4" s="63" t="inlineStr">
         <is>
           <t>การถูกบังคับให้ขายตอนตลาดลง คือสาเหตุอันดับ 1 ของการขาดทุนถาวร</t>
         </is>
@@ -28081,15 +28093,15 @@
       </c>
     </row>
     <row r="5" ht="34" customHeight="1">
-      <c r="A5" s="50" t="n">
+      <c r="A5" s="51" t="n">
         <v>2</v>
       </c>
-      <c r="B5" s="61" t="inlineStr">
+      <c r="B5" s="62" t="inlineStr">
         <is>
           <t>เงินสำรอง 6 เดือนต้องเต็มก่อน จึงจะซื้อสินทรัพย์ชั้น 3 ได้</t>
         </is>
       </c>
-      <c r="C5" s="62" t="inlineStr">
+      <c r="C5" s="63" t="inlineStr">
         <is>
           <t>รายได้นายหน้าไม่สม่ำเสมอ · เงินสำรองคือสิ่งที่ทำให้คุณไม่ต้องขายของถูก</t>
         </is>
@@ -28101,15 +28113,15 @@
       </c>
     </row>
     <row r="6" ht="34" customHeight="1">
-      <c r="A6" s="50" t="n">
+      <c r="A6" s="51" t="n">
         <v>3</v>
       </c>
-      <c r="B6" s="61" t="inlineStr">
+      <c r="B6" s="62" t="inlineStr">
         <is>
           <t>ห้ามใช้เงินกู้ บัตรเครดิต หรือมาร์จิ้น มาลงทุนหรือมาเติมค่าโฆษณา</t>
         </is>
       </c>
-      <c r="C6" s="62" t="inlineStr">
+      <c r="C6" s="63" t="inlineStr">
         <is>
           <t>หนี้เปลี่ยนการขาดทุนชั่วคราวให้กลายเป็นการล้มละลายถาวร</t>
         </is>
@@ -28121,15 +28133,15 @@
       </c>
     </row>
     <row r="7" ht="34" customHeight="1">
-      <c r="A7" s="50" t="n">
+      <c r="A7" s="51" t="n">
         <v>4</v>
       </c>
-      <c r="B7" s="61" t="inlineStr">
+      <c r="B7" s="62" t="inlineStr">
         <is>
           <t>ห้ามใส่เงินเกิน 10% ของพอร์ตในสินทรัพย์ตัวเดียว (ยกเว้นชั้น 0-1)</t>
         </is>
       </c>
-      <c r="C7" s="62" t="inlineStr">
+      <c r="C7" s="63" t="inlineStr">
         <is>
           <t>บริษัทเดียวล้มได้ · ตลาดทั้งตลาดล้มยากกว่ามาก</t>
         </is>
@@ -28141,15 +28153,15 @@
       </c>
     </row>
     <row r="8" ht="34" customHeight="1">
-      <c r="A8" s="50" t="n">
+      <c r="A8" s="51" t="n">
         <v>5</v>
       </c>
-      <c r="B8" s="61" t="inlineStr">
+      <c r="B8" s="62" t="inlineStr">
         <is>
           <t>เพิ่มงบโฆษณาได้เฉพาะเมื่อ ROAS 30 วัน ≥ 3 เท่า และเพิ่มครั้งละไม่เกิน 20%</t>
         </is>
       </c>
-      <c r="C8" s="62" t="inlineStr">
+      <c r="C8" s="63" t="inlineStr">
         <is>
           <t>การเพิ่มงบตอนตัวเลขยังไม่นิ่ง คือการเร่งเผาเงินให้เร็วขึ้น</t>
         </is>
@@ -28161,15 +28173,15 @@
       </c>
     </row>
     <row r="9" ht="34" customHeight="1">
-      <c r="A9" s="50" t="n">
+      <c r="A9" s="51" t="n">
         <v>6</v>
       </c>
-      <c r="B9" s="61" t="inlineStr">
+      <c r="B9" s="62" t="inlineStr">
         <is>
           <t>ถ้า CPQL 7 วันเกินเพดาน 2 วันติด ให้หยุดแอด แล้วแก้คอนเทนต์/กลุ่มเป้าหมายก่อน</t>
         </is>
       </c>
-      <c r="C9" s="62" t="inlineStr">
+      <c r="C9" s="63" t="inlineStr">
         <is>
           <t>เพดานคือเบรกที่คำนวณจากกำไรจริง ไม่ใช่ความรู้สึก</t>
         </is>
@@ -28181,15 +28193,15 @@
       </c>
     </row>
     <row r="10" ht="34" customHeight="1">
-      <c r="A10" s="50" t="n">
+      <c r="A10" s="51" t="n">
         <v>7</v>
       </c>
-      <c r="B10" s="61" t="inlineStr">
+      <c r="B10" s="62" t="inlineStr">
         <is>
           <t>ห้ามซื้อ-ขายตามข่าว กลุ่มไลน์ หรือคนแนะนำ — ซื้อตามแผน DCA เท่านั้น</t>
         </is>
       </c>
-      <c r="C10" s="62" t="inlineStr">
+      <c r="C10" s="63" t="inlineStr">
         <is>
           <t>การจับจังหวะตลาดแพ้ DCA ในระยะยาวเกือบทุกกรณี และกินเวลาสมองที่ควรใช้กับธุรกิจ</t>
         </is>
@@ -28201,15 +28213,15 @@
       </c>
     </row>
     <row r="11" ht="34" customHeight="1">
-      <c r="A11" s="50" t="n">
+      <c r="A11" s="51" t="n">
         <v>8</v>
       </c>
-      <c r="B11" s="61" t="inlineStr">
+      <c r="B11" s="62" t="inlineStr">
         <is>
           <t>Rebalance ปีละ 2 ครั้ง (มิ.ย. และ ธ.ค.) หรือเมื่อชั้นใดเบี่ยงเกิน 5%</t>
         </is>
       </c>
-      <c r="C11" s="62" t="inlineStr">
+      <c r="C11" s="63" t="inlineStr">
         <is>
           <t>บังคับให้ 'ขายของที่ขึ้น ซื้อของที่ลง' โดยอัตโนมัติ โดยไม่ต้องใช้อารมณ์</t>
         </is>
@@ -28221,15 +28233,15 @@
       </c>
     </row>
     <row r="12" ht="34" customHeight="1">
-      <c r="A12" s="50" t="n">
+      <c r="A12" s="51" t="n">
         <v>9</v>
       </c>
-      <c r="B12" s="61" t="inlineStr">
+      <c r="B12" s="62" t="inlineStr">
         <is>
           <t>อะไรที่การันตีผลตอบแทนเกิน 10% ต่อเดือน = แชร์ลูกโซ่ 100% ปฏิเสธทันที</t>
         </is>
       </c>
-      <c r="C12" s="62" t="inlineStr">
+      <c r="C12" s="63" t="inlineStr">
         <is>
           <t>ไม่มีข้อยกเว้น ไม่มี 'รอบนี้พิเศษ' · ตรวจใบอนุญาตที่ SEC Check First ก่อนโอนเงินทุกครั้ง</t>
         </is>
@@ -28241,15 +28253,15 @@
       </c>
     </row>
     <row r="13" ht="34" customHeight="1">
-      <c r="A13" s="50" t="n">
+      <c r="A13" s="51" t="n">
         <v>10</v>
       </c>
-      <c r="B13" s="61" t="inlineStr">
+      <c r="B13" s="62" t="inlineStr">
         <is>
           <t>บันทึกตัวเลขทุกวันก่อน 21:00 น. ไม่มีข้อยกเว้น</t>
         </is>
       </c>
-      <c r="C13" s="62" t="inlineStr">
+      <c r="C13" s="63" t="inlineStr">
         <is>
           <t>สิ่งที่ไม่ได้วัด จะไม่มีทางดีขึ้น · 3 นาที/วัน คือราคาที่ถูกที่สุดของความสำเร็จ</t>
         </is>
@@ -28261,15 +28273,15 @@
       </c>
     </row>
     <row r="14" ht="34" customHeight="1">
-      <c r="A14" s="50" t="n">
+      <c r="A14" s="51" t="n">
         <v>11</v>
       </c>
-      <c r="B14" s="61" t="inlineStr">
+      <c r="B14" s="62" t="inlineStr">
         <is>
           <t>โอนกำไรเข้าพอร์ตทุกวันที่ 1 และ 16 — ก่อนใช้จ่ายอย่างอื่น</t>
         </is>
       </c>
-      <c r="C14" s="62" t="inlineStr">
+      <c r="C14" s="63" t="inlineStr">
         <is>
           <t>จ่ายให้ตัวเองก่อนเสมอ · เงินที่เหลือค่อยใช้ ไม่ใช่ใช้แล้วค่อยเหลือ</t>
         </is>
@@ -28281,15 +28293,15 @@
       </c>
     </row>
     <row r="15" ht="34" customHeight="1">
-      <c r="A15" s="50" t="n">
+      <c r="A15" s="51" t="n">
         <v>12</v>
       </c>
-      <c r="B15" s="61" t="inlineStr">
+      <c r="B15" s="62" t="inlineStr">
         <is>
           <t>แยกบัญชีธนาคาร 4 ใบจริง: ธุรกิจ / ภาษี+สำรอง / ลงทุน / ใช้จ่าย</t>
         </is>
       </c>
-      <c r="C15" s="62" t="inlineStr">
+      <c r="C15" s="63" t="inlineStr">
         <is>
           <t>ระบบชนะวินัย · ถ้าเงินอยู่กองเดียวกัน มันจะถูกใช้หมดเสมอ</t>
         </is>
@@ -28301,15 +28313,15 @@
       </c>
     </row>
     <row r="16" ht="34" customHeight="1">
-      <c r="A16" s="50" t="n">
+      <c r="A16" s="51" t="n">
         <v>13</v>
       </c>
-      <c r="B16" s="61" t="inlineStr">
+      <c r="B16" s="62" t="inlineStr">
         <is>
           <t>กันภาษี 30% ของค่าคอมทันทีที่ได้รับ</t>
         </is>
       </c>
-      <c r="C16" s="62" t="inlineStr">
+      <c r="C16" s="63" t="inlineStr">
         <is>
           <t>นายหน้าถูกหัก ณ ที่จ่ายไม่ครบ ต้องยื่นเพิ่มปลายปี · คนที่ลืมกันภาษีคือคนที่เจ็บที่สุดในเดือนมีนาคม</t>
         </is>
@@ -28321,15 +28333,15 @@
       </c>
     </row>
     <row r="17" ht="34" customHeight="1">
-      <c r="A17" s="50" t="n">
+      <c r="A17" s="51" t="n">
         <v>14</v>
       </c>
-      <c r="B17" s="61" t="inlineStr">
+      <c r="B17" s="62" t="inlineStr">
         <is>
           <t>ตรวจเอกสารสิทธิ์ ผู้ขาย และใบอนุญาตโครงการทุกดีล ก่อนพาลูกค้าดู</t>
         </is>
       </c>
-      <c r="C17" s="62" t="inlineStr">
+      <c r="C17" s="63" t="inlineStr">
         <is>
           <t>ดีลเดียวที่มีปัญหาทางกฎหมาย ลบกำไรทั้งปีได้ และเสียชื่อถาวรในตลาดเล็กอย่างหาดใหญ่</t>
         </is>
@@ -28341,15 +28353,15 @@
       </c>
     </row>
     <row r="18" ht="34" customHeight="1">
-      <c r="A18" s="50" t="n">
+      <c r="A18" s="51" t="n">
         <v>15</v>
       </c>
-      <c r="B18" s="61" t="inlineStr">
+      <c r="B18" s="62" t="inlineStr">
         <is>
           <t>พอร์ตติดลบเกิน 20% → ห้ามขาย ห้ามหยุด DCA ให้ซื้อต่อตามแผนเดิม</t>
         </is>
       </c>
-      <c r="C18" s="62" t="inlineStr">
+      <c r="C18" s="63" t="inlineStr">
         <is>
           <t>ช่วงที่เจ็บที่สุด คือช่วงที่ราคาถูกที่สุด · แผนเขียนไว้ตอนใจนิ่ง ให้เชื่อแผน ไม่ใช่เชื่อใจตอนตกใจ</t>
         </is>
@@ -28469,484 +28481,484 @@
       </c>
     </row>
     <row r="4" ht="30" customHeight="1">
-      <c r="A4" s="63" t="n">
+      <c r="A4" s="64" t="n">
         <v>46266</v>
       </c>
-      <c r="B4" s="64" t="n">
+      <c r="B4" s="65" t="n">
         <v>1</v>
       </c>
-      <c r="C4" s="51">
+      <c r="C4" s="52">
         <f>ROUND(B4*'ตั้งค่า'!$C$8,0)</f>
         <v/>
       </c>
-      <c r="D4" s="51">
+      <c r="D4" s="52">
         <f>ROUND(MAX('ตั้งค่า'!$C$21,C4*0.15),0)</f>
         <v/>
       </c>
-      <c r="E4" s="51">
+      <c r="E4" s="52">
         <f>'ตั้งค่า'!$C$10</f>
         <v/>
       </c>
-      <c r="F4" s="51">
+      <c r="F4" s="52">
         <f>C4-D4-E4</f>
         <v/>
       </c>
-      <c r="G4" s="51">
+      <c r="G4" s="52">
         <f>ROUND(C4*'ตั้งค่า'!$C$36,0)</f>
         <v/>
       </c>
-      <c r="H4" s="55">
+      <c r="H4" s="56">
         <f>ROUND('ตั้งค่า'!$C$28*(1+'ตั้งค่า'!$C$49/12)+G4,0)</f>
         <v/>
       </c>
-      <c r="I4" s="65" t="inlineStr">
+      <c r="I4" s="66" t="inlineStr">
         <is>
           <t>ตั้งระบบ: แยกบัญชี 4 ใบ · เริ่มบันทึกทุกวัน · เติมเงินสำรองเป็นอันดับแรก</t>
         </is>
       </c>
     </row>
     <row r="5" ht="30" customHeight="1">
-      <c r="A5" s="63" t="n">
+      <c r="A5" s="64" t="n">
         <v>46296</v>
       </c>
-      <c r="B5" s="64" t="n">
+      <c r="B5" s="65" t="n">
         <v>1</v>
       </c>
-      <c r="C5" s="51">
+      <c r="C5" s="52">
         <f>ROUND(B5*'ตั้งค่า'!$C$8,0)</f>
         <v/>
       </c>
-      <c r="D5" s="51">
+      <c r="D5" s="52">
         <f>ROUND(MAX('ตั้งค่า'!$C$21,C5*0.15),0)</f>
         <v/>
       </c>
-      <c r="E5" s="51">
+      <c r="E5" s="52">
         <f>'ตั้งค่า'!$C$10</f>
         <v/>
       </c>
-      <c r="F5" s="51">
+      <c r="F5" s="52">
         <f>C5-D5-E5</f>
         <v/>
       </c>
-      <c r="G5" s="51">
+      <c r="G5" s="52">
         <f>ROUND(C5*'ตั้งค่า'!$C$36,0)</f>
         <v/>
       </c>
-      <c r="H5" s="55">
+      <c r="H5" s="56">
         <f>ROUND(H4*(1+'ตั้งค่า'!$C$49/12)+G5,0)</f>
         <v/>
       </c>
-      <c r="I5" s="65" t="inlineStr">
+      <c r="I5" s="66" t="inlineStr">
         <is>
           <t>หา CPQL จริงของตัวเอง: ทดสอบคอนเทนต์ 3 แบบ วัดผลครบ 30 วัน แล้วแก้สมมติฐาน</t>
         </is>
       </c>
     </row>
     <row r="6" ht="30" customHeight="1">
-      <c r="A6" s="63" t="n">
+      <c r="A6" s="64" t="n">
         <v>46327</v>
       </c>
-      <c r="B6" s="64" t="n">
+      <c r="B6" s="65" t="n">
         <v>2</v>
       </c>
-      <c r="C6" s="51">
+      <c r="C6" s="52">
         <f>ROUND(B6*'ตั้งค่า'!$C$8,0)</f>
         <v/>
       </c>
-      <c r="D6" s="51">
+      <c r="D6" s="52">
         <f>ROUND(MAX('ตั้งค่า'!$C$21,C6*0.15),0)</f>
         <v/>
       </c>
-      <c r="E6" s="51">
+      <c r="E6" s="52">
         <f>'ตั้งค่า'!$C$10</f>
         <v/>
       </c>
-      <c r="F6" s="51">
+      <c r="F6" s="52">
         <f>C6-D6-E6</f>
         <v/>
       </c>
-      <c r="G6" s="51">
+      <c r="G6" s="52">
         <f>ROUND(C6*'ตั้งค่า'!$C$36,0)</f>
         <v/>
       </c>
-      <c r="H6" s="55">
+      <c r="H6" s="56">
         <f>ROUND(H5*(1+'ตั้งค่า'!$C$49/12)+G6,0)</f>
         <v/>
       </c>
-      <c r="I6" s="65" t="inlineStr">
+      <c r="I6" s="66" t="inlineStr">
         <is>
           <t>เติม FAQ ใน Google Sheet ของ LINE bot ให้ครบ 50 คำถาม — ลดเวลาตอบ เพิ่มจำนวน lead ที่รับไหว</t>
         </is>
       </c>
     </row>
     <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="63" t="n">
+      <c r="A7" s="64" t="n">
         <v>46357</v>
       </c>
-      <c r="B7" s="64" t="n">
+      <c r="B7" s="65" t="n">
         <v>2</v>
       </c>
-      <c r="C7" s="51">
+      <c r="C7" s="52">
         <f>ROUND(B7*'ตั้งค่า'!$C$8,0)</f>
         <v/>
       </c>
-      <c r="D7" s="51">
+      <c r="D7" s="52">
         <f>ROUND(MAX('ตั้งค่า'!$C$21,C7*0.15),0)</f>
         <v/>
       </c>
-      <c r="E7" s="51">
+      <c r="E7" s="52">
         <f>'ตั้งค่า'!$C$10</f>
         <v/>
       </c>
-      <c r="F7" s="51">
+      <c r="F7" s="52">
         <f>C7-D7-E7</f>
         <v/>
       </c>
-      <c r="G7" s="51">
+      <c r="G7" s="52">
         <f>ROUND(C7*'ตั้งค่า'!$C$36,0)</f>
         <v/>
       </c>
-      <c r="H7" s="55">
+      <c r="H7" s="56">
         <f>ROUND(H6*(1+'ตั้งค่า'!$C$49/12)+G7,0)</f>
         <v/>
       </c>
-      <c r="I7" s="65" t="inlineStr">
+      <c r="I7" s="66" t="inlineStr">
         <is>
           <t>เงินสำรองควรเต็มครึ่งทาง · เริ่มซื้อชั้น 1 (พันธบัตร/กองตราสารหนี้)</t>
         </is>
       </c>
     </row>
     <row r="8" ht="30" customHeight="1">
-      <c r="A8" s="63" t="n">
+      <c r="A8" s="64" t="n">
         <v>46388</v>
       </c>
-      <c r="B8" s="64" t="n">
+      <c r="B8" s="65" t="n">
         <v>2</v>
       </c>
-      <c r="C8" s="51">
+      <c r="C8" s="52">
         <f>ROUND(B8*'ตั้งค่า'!$C$8,0)</f>
         <v/>
       </c>
-      <c r="D8" s="51">
+      <c r="D8" s="52">
         <f>ROUND(MAX('ตั้งค่า'!$C$21,C8*0.15),0)</f>
         <v/>
       </c>
-      <c r="E8" s="51">
+      <c r="E8" s="52">
         <f>'ตั้งค่า'!$C$10</f>
         <v/>
       </c>
-      <c r="F8" s="51">
+      <c r="F8" s="52">
         <f>C8-D8-E8</f>
         <v/>
       </c>
-      <c r="G8" s="51">
+      <c r="G8" s="52">
         <f>ROUND(C8*'ตั้งค่า'!$C$36,0)</f>
         <v/>
       </c>
-      <c r="H8" s="55">
+      <c r="H8" s="56">
         <f>ROUND(H7*(1+'ตั้งค่า'!$C$49/12)+G8,0)</f>
         <v/>
       </c>
-      <c r="I8" s="65" t="inlineStr">
+      <c r="I8" s="66" t="inlineStr">
         <is>
           <t>เก็บรีวิวลูกค้าจริง 5 ราย ทำเป็นคอนเทนต์ — รีวิวจริงคือสิ่งที่ลด CPQL ได้มากที่สุด</t>
         </is>
       </c>
     </row>
     <row r="9" ht="30" customHeight="1">
-      <c r="A9" s="63" t="n">
+      <c r="A9" s="64" t="n">
         <v>46419</v>
       </c>
-      <c r="B9" s="64" t="n">
+      <c r="B9" s="65" t="n">
         <v>3</v>
       </c>
-      <c r="C9" s="51">
+      <c r="C9" s="52">
         <f>ROUND(B9*'ตั้งค่า'!$C$8,0)</f>
         <v/>
       </c>
-      <c r="D9" s="51">
+      <c r="D9" s="52">
         <f>ROUND(MAX('ตั้งค่า'!$C$21,C9*0.15),0)</f>
         <v/>
       </c>
-      <c r="E9" s="51">
+      <c r="E9" s="52">
         <f>'ตั้งค่า'!$C$10</f>
         <v/>
       </c>
-      <c r="F9" s="51">
+      <c r="F9" s="52">
         <f>C9-D9-E9</f>
         <v/>
       </c>
-      <c r="G9" s="51">
+      <c r="G9" s="52">
         <f>ROUND(C9*'ตั้งค่า'!$C$36,0)</f>
         <v/>
       </c>
-      <c r="H9" s="55">
+      <c r="H9" s="56">
         <f>ROUND(H8*(1+'ตั้งค่า'!$C$49/12)+G9,0)</f>
         <v/>
       </c>
-      <c r="I9" s="65" t="inlineStr">
+      <c r="I9" s="66" t="inlineStr">
         <is>
           <t>ทบทวนครึ่งปี: แก้ทุกสมมติฐานด้วยตัวเลขจริง · Rebalance ครั้งที่ 1</t>
         </is>
       </c>
     </row>
     <row r="10" ht="30" customHeight="1">
-      <c r="A10" s="63" t="n">
+      <c r="A10" s="64" t="n">
         <v>46447</v>
       </c>
-      <c r="B10" s="64" t="n">
+      <c r="B10" s="65" t="n">
         <v>3</v>
       </c>
-      <c r="C10" s="51">
+      <c r="C10" s="52">
         <f>ROUND(B10*'ตั้งค่า'!$C$8,0)</f>
         <v/>
       </c>
-      <c r="D10" s="51">
+      <c r="D10" s="52">
         <f>ROUND(MAX('ตั้งค่า'!$C$21,C10*0.15),0)</f>
         <v/>
       </c>
-      <c r="E10" s="51">
+      <c r="E10" s="52">
         <f>'ตั้งค่า'!$C$10</f>
         <v/>
       </c>
-      <c r="F10" s="51">
+      <c r="F10" s="52">
         <f>C10-D10-E10</f>
         <v/>
       </c>
-      <c r="G10" s="51">
+      <c r="G10" s="52">
         <f>ROUND(C10*'ตั้งค่า'!$C$36,0)</f>
         <v/>
       </c>
-      <c r="H10" s="55">
+      <c r="H10" s="56">
         <f>ROUND(H9*(1+'ตั้งค่า'!$C$49/12)+G10,0)</f>
         <v/>
       </c>
-      <c r="I10" s="65" t="inlineStr">
+      <c r="I10" s="66" t="inlineStr">
         <is>
           <t>เงินสำรองเต็ม 100% → เริ่มชั้น 2 (หุ้นกู้เรตติ้งดี / REIT)</t>
         </is>
       </c>
     </row>
     <row r="11" ht="30" customHeight="1">
-      <c r="A11" s="63" t="n">
+      <c r="A11" s="64" t="n">
         <v>46478</v>
       </c>
-      <c r="B11" s="64" t="n">
+      <c r="B11" s="65" t="n">
         <v>3</v>
       </c>
-      <c r="C11" s="51">
+      <c r="C11" s="52">
         <f>ROUND(B11*'ตั้งค่า'!$C$8,0)</f>
         <v/>
       </c>
-      <c r="D11" s="51">
+      <c r="D11" s="52">
         <f>ROUND(MAX('ตั้งค่า'!$C$21,C11*0.15),0)</f>
         <v/>
       </c>
-      <c r="E11" s="51">
+      <c r="E11" s="52">
         <f>'ตั้งค่า'!$C$10</f>
         <v/>
       </c>
-      <c r="F11" s="51">
+      <c r="F11" s="52">
         <f>C11-D11-E11</f>
         <v/>
       </c>
-      <c r="G11" s="51">
+      <c r="G11" s="52">
         <f>ROUND(C11*'ตั้งค่า'!$C$36,0)</f>
         <v/>
       </c>
-      <c r="H11" s="55">
+      <c r="H11" s="56">
         <f>ROUND(H10*(1+'ตั้งค่า'!$C$49/12)+G11,0)</f>
         <v/>
       </c>
-      <c r="I11" s="65" t="inlineStr">
+      <c r="I11" s="66" t="inlineStr">
         <is>
           <t>ขยายทรัพย์ในมือ: เซ็นสัญญานายหน้ากับเจ้าของบ้าน/โครงการเพิ่มอีก 10 รายการ</t>
         </is>
       </c>
     </row>
     <row r="12" ht="30" customHeight="1">
-      <c r="A12" s="63" t="n">
+      <c r="A12" s="64" t="n">
         <v>46508</v>
       </c>
-      <c r="B12" s="64" t="n">
+      <c r="B12" s="65" t="n">
         <v>4</v>
       </c>
-      <c r="C12" s="51">
+      <c r="C12" s="52">
         <f>ROUND(B12*'ตั้งค่า'!$C$8,0)</f>
         <v/>
       </c>
-      <c r="D12" s="51">
+      <c r="D12" s="52">
         <f>ROUND(MAX('ตั้งค่า'!$C$21,C12*0.15),0)</f>
         <v/>
       </c>
-      <c r="E12" s="51">
+      <c r="E12" s="52">
         <f>'ตั้งค่า'!$C$10</f>
         <v/>
       </c>
-      <c r="F12" s="51">
+      <c r="F12" s="52">
         <f>C12-D12-E12</f>
         <v/>
       </c>
-      <c r="G12" s="51">
+      <c r="G12" s="52">
         <f>ROUND(C12*'ตั้งค่า'!$C$36,0)</f>
         <v/>
       </c>
-      <c r="H12" s="55">
+      <c r="H12" s="56">
         <f>ROUND(H11*(1+'ตั้งค่า'!$C$49/12)+G12,0)</f>
         <v/>
       </c>
-      <c r="I12" s="65" t="inlineStr">
+      <c r="I12" s="66" t="inlineStr">
         <is>
           <t>เริ่ม DCA ชั้น 3 (กองดัชนีหุ้นโลก) ทุกวันที่ 1 · ตั้งคำสั่งซื้ออัตโนมัติ จะได้ไม่ต้องใช้ใจ</t>
         </is>
       </c>
     </row>
     <row r="13" ht="30" customHeight="1">
-      <c r="A13" s="63" t="n">
+      <c r="A13" s="64" t="n">
         <v>46539</v>
       </c>
-      <c r="B13" s="64" t="n">
+      <c r="B13" s="65" t="n">
         <v>4</v>
       </c>
-      <c r="C13" s="51">
+      <c r="C13" s="52">
         <f>ROUND(B13*'ตั้งค่า'!$C$8,0)</f>
         <v/>
       </c>
-      <c r="D13" s="51">
+      <c r="D13" s="52">
         <f>ROUND(MAX('ตั้งค่า'!$C$21,C13*0.15),0)</f>
         <v/>
       </c>
-      <c r="E13" s="51">
+      <c r="E13" s="52">
         <f>'ตั้งค่า'!$C$10</f>
         <v/>
       </c>
-      <c r="F13" s="51">
+      <c r="F13" s="52">
         <f>C13-D13-E13</f>
         <v/>
       </c>
-      <c r="G13" s="51">
+      <c r="G13" s="52">
         <f>ROUND(C13*'ตั้งค่า'!$C$36,0)</f>
         <v/>
       </c>
-      <c r="H13" s="55">
+      <c r="H13" s="56">
         <f>ROUND(H12*(1+'ตั้งค่า'!$C$49/12)+G13,0)</f>
         <v/>
       </c>
-      <c r="I13" s="65" t="inlineStr">
+      <c r="I13" s="66" t="inlineStr">
         <is>
           <t>หาผู้ช่วยตอบแชท 1 คน — คอขวดของธุรกิจนี้คือเวลาตอบ ไม่ใช่จำนวน lead</t>
         </is>
       </c>
     </row>
     <row r="14" ht="30" customHeight="1">
-      <c r="A14" s="63" t="n">
+      <c r="A14" s="64" t="n">
         <v>46569</v>
       </c>
-      <c r="B14" s="64" t="n">
+      <c r="B14" s="65" t="n">
         <v>4</v>
       </c>
-      <c r="C14" s="51">
+      <c r="C14" s="52">
         <f>ROUND(B14*'ตั้งค่า'!$C$8,0)</f>
         <v/>
       </c>
-      <c r="D14" s="51">
+      <c r="D14" s="52">
         <f>ROUND(MAX('ตั้งค่า'!$C$21,C14*0.15),0)</f>
         <v/>
       </c>
-      <c r="E14" s="51">
+      <c r="E14" s="52">
         <f>'ตั้งค่า'!$C$10</f>
         <v/>
       </c>
-      <c r="F14" s="51">
+      <c r="F14" s="52">
         <f>C14-D14-E14</f>
         <v/>
       </c>
-      <c r="G14" s="51">
+      <c r="G14" s="52">
         <f>ROUND(C14*'ตั้งค่า'!$C$36,0)</f>
         <v/>
       </c>
-      <c r="H14" s="55">
+      <c r="H14" s="56">
         <f>ROUND(H13*(1+'ตั้งค่า'!$C$49/12)+G14,0)</f>
         <v/>
       </c>
-      <c r="I14" s="65" t="inlineStr">
+      <c r="I14" s="66" t="inlineStr">
         <is>
           <t>วางแผนภาษีปลายปี: ซื้อกองลดหย่อน (ชั้น 4) ให้เต็มสิทธิ์ก่อน 31 ธ.ค.</t>
         </is>
       </c>
     </row>
     <row r="15" ht="30" customHeight="1">
-      <c r="A15" s="63" t="n">
+      <c r="A15" s="64" t="n">
         <v>46600</v>
       </c>
-      <c r="B15" s="64" t="n">
+      <c r="B15" s="65" t="n">
         <v>5</v>
       </c>
-      <c r="C15" s="51">
+      <c r="C15" s="52">
         <f>ROUND(B15*'ตั้งค่า'!$C$8,0)</f>
         <v/>
       </c>
-      <c r="D15" s="51">
+      <c r="D15" s="52">
         <f>ROUND(MAX('ตั้งค่า'!$C$21,C15*0.15),0)</f>
         <v/>
       </c>
-      <c r="E15" s="51">
+      <c r="E15" s="52">
         <f>'ตั้งค่า'!$C$10</f>
         <v/>
       </c>
-      <c r="F15" s="51">
+      <c r="F15" s="52">
         <f>C15-D15-E15</f>
         <v/>
       </c>
-      <c r="G15" s="51">
+      <c r="G15" s="52">
         <f>ROUND(C15*'ตั้งค่า'!$C$36,0)</f>
         <v/>
       </c>
-      <c r="H15" s="55">
+      <c r="H15" s="56">
         <f>ROUND(H14*(1+'ตั้งค่า'!$C$49/12)+G15,0)</f>
         <v/>
       </c>
-      <c r="I15" s="65" t="inlineStr">
+      <c r="I15" s="66" t="inlineStr">
         <is>
           <t>ปิดปี: สรุปตัวเลขจริงทั้งปี · Rebalance ครั้งที่ 2 · ตั้งเป้าปีหน้าจากของจริง ไม่ใช่จากความหวัง</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="44" t="inlineStr">
+      <c r="A16" s="45" t="inlineStr">
         <is>
           <t>รวม 12 เดือน</t>
         </is>
       </c>
-      <c r="B16" s="66">
+      <c r="B16" s="67">
         <f>SUM(B4:B15)</f>
         <v/>
       </c>
-      <c r="C16" s="46">
+      <c r="C16" s="47">
         <f>SUM(C4:C15)</f>
         <v/>
       </c>
-      <c r="D16" s="46">
+      <c r="D16" s="47">
         <f>SUM(D4:D15)</f>
         <v/>
       </c>
-      <c r="E16" s="46">
+      <c r="E16" s="47">
         <f>SUM(E4:E15)</f>
         <v/>
       </c>
-      <c r="F16" s="46">
+      <c r="F16" s="47">
         <f>SUM(F4:F15)</f>
         <v/>
       </c>
-      <c r="G16" s="46">
+      <c r="G16" s="47">
         <f>SUM(G4:G15)</f>
         <v/>
       </c>
-      <c r="H16" s="46">
+      <c r="H16" s="47">
         <f>H15</f>
         <v/>
       </c>
-      <c r="I16" s="67" t="inlineStr">
+      <c r="I16" s="68" t="inlineStr">
         <is>
           <t>มูลค่าพอร์ตปลายปีที่ 1 (ประมาณการ)</t>
         </is>

</xml_diff>